<commit_message>
fix: La Caixa parser - match real format "ON 36XXXXXXX DDMM"
The bank statement uses "ON " + terminal number (first 2 digits = license)
instead of compact "ON34/ON35/ON36". Also handles "C." correction entries.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/lacaixa_sample.xlsx
+++ b/tests/fixtures/lacaixa_sample.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Moviments" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Moviments_compte" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -416,13 +416,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Moviments del compte ES12 3456 7890 1234 5678</t>
+          <t>Moviments del compte ES73 2100 3000 1722 0245 8470</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Imports expressats en euros</t>
         </is>
       </c>
     </row>
@@ -444,7 +451,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Mes dades</t>
+          <t>Més dades</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -463,18 +470,14 @@
         <v>46049</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>46050</v>
+        <v>46049</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ON34 TPV COBRO</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Cobro TPV taxi</t>
-        </is>
-      </c>
+          <t>ON 340921234 2601</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
         <v>152.3</v>
       </c>
@@ -484,26 +487,22 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46049</v>
+        <v>46050</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>46050</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ON35 TPV COBRO</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Cobro TPV taxi</t>
-        </is>
-      </c>
+          <t>ON 340921234 2701</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>89.5</v>
+        <v>98.75</v>
       </c>
       <c r="F5" t="n">
-        <v>5089.5</v>
+        <v>5098.75</v>
       </c>
     </row>
     <row r="6">
@@ -511,23 +510,19 @@
         <v>46050</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>46051</v>
+        <v>46050</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ON36 TPV COBRO</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Cobro TPV taxi</t>
-        </is>
-      </c>
+          <t>ON 351061567 2701</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
-        <v>210</v>
+        <v>89.5</v>
       </c>
       <c r="F6" t="n">
-        <v>5299.5</v>
+        <v>5188.25</v>
       </c>
     </row>
     <row r="7">
@@ -535,47 +530,63 @@
         <v>46050</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>46051</v>
+        <v>46050</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>TRANSFERENCIA</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Transferencia recibida</t>
-        </is>
-      </c>
+          <t>ON 363460767 2701</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
-        <v>500</v>
+        <v>111.65</v>
       </c>
       <c r="F7" t="n">
-        <v>5799.5</v>
+        <v>5299.9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46051</v>
+        <v>46050</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>46052</v>
+        <v>46050</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ON34 TPV COBRO</t>
+          <t>TRANSF AL SEU FAVOR</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Cobro TPV taxi</t>
+          <t>MYTAXI IBERIA SL.</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>75</v>
+        <v>264.02</v>
       </c>
       <c r="F8" t="n">
-        <v>5874.5</v>
+        <v>5563.92</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>46049</v>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>46049</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>C. 363460767 2601</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="n">
+        <v>-0.13</v>
+      </c>
+      <c r="F9" t="n">
+        <v>5563.79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>